<commit_message>
added lots of cds
de 97 para 115? bues cds mesmo
</commit_message>
<xml_diff>
--- a/albums.xlsx
+++ b/albums.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\site\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5561AD29-066D-4331-819B-AC946EE69C8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9D4B8B5-4098-457E-8522-5B63ECDD8DA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5124" yWindow="336" windowWidth="25380" windowHeight="17616" xr2:uid="{53D4B46E-FDBF-49C0-B10D-66A1716C0584}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="330">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="386">
   <si>
     <t>Goldie</t>
   </si>
@@ -1015,6 +1015,174 @@
   </si>
   <si>
     <t>Quality Records</t>
+  </si>
+  <si>
+    <t>c115</t>
+  </si>
+  <si>
+    <t>c114</t>
+  </si>
+  <si>
+    <t>c113</t>
+  </si>
+  <si>
+    <t>c112</t>
+  </si>
+  <si>
+    <t>c111</t>
+  </si>
+  <si>
+    <t>c110</t>
+  </si>
+  <si>
+    <t>c109</t>
+  </si>
+  <si>
+    <t>c108</t>
+  </si>
+  <si>
+    <t>c107</t>
+  </si>
+  <si>
+    <t>c106</t>
+  </si>
+  <si>
+    <t>c105</t>
+  </si>
+  <si>
+    <t>c104</t>
+  </si>
+  <si>
+    <t>c103</t>
+  </si>
+  <si>
+    <t>c102</t>
+  </si>
+  <si>
+    <t>c101</t>
+  </si>
+  <si>
+    <t>c100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boymerang </t>
+  </si>
+  <si>
+    <t>Balance of the Force</t>
+  </si>
+  <si>
+    <t>Astrelworks</t>
+  </si>
+  <si>
+    <t>Omni Trio</t>
+  </si>
+  <si>
+    <t>Haunted Science</t>
+  </si>
+  <si>
+    <t>Moving Shadow</t>
+  </si>
+  <si>
+    <t>Human Traffic (Essential Selection Presents Music From The Motion Picture)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ohm G </t>
+  </si>
+  <si>
+    <t>Future Ballads</t>
+  </si>
+  <si>
+    <t>Jubilee Records</t>
+  </si>
+  <si>
+    <t>Bazille Noir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bazille Noir </t>
+  </si>
+  <si>
+    <t>Markus Kienzl</t>
+  </si>
+  <si>
+    <t>Tilt EP</t>
+  </si>
+  <si>
+    <t>Klein Records</t>
+  </si>
+  <si>
+    <t>Sofa Surfers</t>
+  </si>
+  <si>
+    <t>Cargo</t>
+  </si>
+  <si>
+    <t>Talvin Singh</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>Island Records</t>
+  </si>
+  <si>
+    <t>覚醒 - Kakusei</t>
+  </si>
+  <si>
+    <t>DJ Krush</t>
+  </si>
+  <si>
+    <t>Sony Music</t>
+  </si>
+  <si>
+    <t>HIPHOP, ELETRONIC</t>
+  </si>
+  <si>
+    <t>Platinum Breakz II</t>
+  </si>
+  <si>
+    <t>Vic Acid</t>
+  </si>
+  <si>
+    <t>Opiate</t>
+  </si>
+  <si>
+    <t>Sometimes</t>
+  </si>
+  <si>
+    <t>Morr Music</t>
+  </si>
+  <si>
+    <t>The Day My Favourite Insect Died</t>
+  </si>
+  <si>
+    <t>Kollaps</t>
+  </si>
+  <si>
+    <t>Source Direct</t>
+  </si>
+  <si>
+    <t>Two Masks / Black Domina</t>
+  </si>
+  <si>
+    <t>SOUNDTRACK, ELETRONIC</t>
+  </si>
+  <si>
+    <t>In The Mood For Love (Original Soundtrack From The Motion Picture)</t>
+  </si>
+  <si>
+    <t>Virgin</t>
+  </si>
+  <si>
+    <t>SOUNDTRACK, CLASSICAL</t>
+  </si>
+  <si>
+    <t>Earthworks</t>
+  </si>
+  <si>
+    <t>ELETRONIC, HIPHOP</t>
+  </si>
+  <si>
+    <t>Kwaito - South African Hip Hop</t>
   </si>
 </sst>
 </file>
@@ -1062,7 +1230,79 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="11">
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125">
+          <fgColor theme="1" tint="4.9989318521683403E-2"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125">
+          <fgColor theme="1" tint="4.9989318521683403E-2"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125">
+          <fgColor theme="1" tint="4.9989318521683403E-2"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125">
+          <fgColor theme="1" tint="4.9989318521683403E-2"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125">
+          <fgColor theme="1" tint="4.9989318521683403E-2"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125">
+          <fgColor theme="1" tint="4.9989318521683403E-2"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125">
+          <fgColor theme="1" tint="4.9989318521683403E-2"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125">
+          <fgColor theme="1" tint="4.9989318521683403E-2"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125">
+          <fgColor theme="1" tint="4.9989318521683403E-2"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="gray125">
@@ -1389,7 +1629,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB66776B-147E-48E9-A2AC-42888F95FB52}">
-  <dimension ref="A1:G97"/>
+  <dimension ref="A1:G113"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24.5546875" bestFit="1" customWidth="1"/>
@@ -1401,22 +1641,22 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="B1" t="s">
-        <v>325</v>
+        <v>3</v>
       </c>
       <c r="C1" t="s">
-        <v>326</v>
+        <v>385</v>
       </c>
       <c r="D1" t="s">
-        <v>327</v>
+        <v>383</v>
       </c>
       <c r="E1">
-        <v>2002</v>
+        <v>2000</v>
       </c>
       <c r="F1" t="s">
-        <v>290</v>
+        <v>384</v>
       </c>
       <c r="G1" t="s">
         <v>241</v>
@@ -1424,22 +1664,22 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>328</v>
+        <v>380</v>
       </c>
       <c r="D2" t="s">
-        <v>329</v>
+        <v>381</v>
       </c>
       <c r="E2">
-        <v>1995</v>
+        <v>2000</v>
       </c>
       <c r="F2" t="s">
-        <v>290</v>
+        <v>382</v>
       </c>
       <c r="G2" t="s">
         <v>241</v>
@@ -1447,19 +1687,19 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>319</v>
+        <v>332</v>
       </c>
       <c r="B3" t="s">
-        <v>321</v>
+        <v>377</v>
       </c>
       <c r="C3" t="s">
-        <v>322</v>
+        <v>378</v>
       </c>
       <c r="D3" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="E3">
-        <v>1995</v>
+        <v>1997</v>
       </c>
       <c r="F3" t="s">
         <v>290</v>
@@ -1470,19 +1710,19 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>318</v>
+        <v>333</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>320</v>
+        <v>375</v>
       </c>
       <c r="D4" t="s">
-        <v>173</v>
+        <v>376</v>
       </c>
       <c r="E4">
-        <v>2001</v>
+        <v>1995</v>
       </c>
       <c r="F4" t="s">
         <v>290</v>
@@ -1493,19 +1733,19 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>306</v>
+        <v>334</v>
       </c>
       <c r="B5" t="s">
-        <v>3</v>
+        <v>372</v>
       </c>
       <c r="C5" t="s">
-        <v>309</v>
+        <v>373</v>
       </c>
       <c r="D5" t="s">
-        <v>310</v>
+        <v>374</v>
       </c>
       <c r="E5">
-        <v>1997</v>
+        <v>2003</v>
       </c>
       <c r="F5" t="s">
         <v>290</v>
@@ -1516,19 +1756,19 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>307</v>
+        <v>335</v>
       </c>
       <c r="B6" t="s">
-        <v>3</v>
+        <v>301</v>
       </c>
       <c r="C6" t="s">
-        <v>311</v>
+        <v>371</v>
       </c>
       <c r="D6" t="s">
-        <v>312</v>
+        <v>173</v>
       </c>
       <c r="E6">
-        <v>1998</v>
+        <v>1997</v>
       </c>
       <c r="F6" t="s">
         <v>290</v>
@@ -1539,19 +1779,19 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>308</v>
+        <v>336</v>
       </c>
       <c r="B7" t="s">
-        <v>313</v>
+        <v>3</v>
       </c>
       <c r="C7" t="s">
-        <v>314</v>
+        <v>370</v>
       </c>
       <c r="D7" t="s">
-        <v>171</v>
+        <v>2</v>
       </c>
       <c r="E7">
-        <v>1996</v>
+        <v>1997</v>
       </c>
       <c r="F7" t="s">
         <v>290</v>
@@ -1562,22 +1802,22 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>305</v>
+        <v>337</v>
       </c>
       <c r="B8" t="s">
-        <v>315</v>
+        <v>367</v>
       </c>
       <c r="C8" t="s">
-        <v>316</v>
+        <v>366</v>
       </c>
       <c r="D8" t="s">
-        <v>317</v>
+        <v>368</v>
       </c>
       <c r="E8">
-        <v>1996</v>
+        <v>1999</v>
       </c>
       <c r="F8" t="s">
-        <v>290</v>
+        <v>369</v>
       </c>
       <c r="G8" t="s">
         <v>241</v>
@@ -1585,19 +1825,19 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>294</v>
+        <v>338</v>
       </c>
       <c r="B9" t="s">
-        <v>301</v>
+        <v>363</v>
       </c>
       <c r="C9" t="s">
-        <v>302</v>
+        <v>364</v>
       </c>
       <c r="D9" t="s">
-        <v>173</v>
+        <v>365</v>
       </c>
       <c r="E9">
-        <v>1999</v>
+        <v>1998</v>
       </c>
       <c r="F9" t="s">
         <v>290</v>
@@ -1608,19 +1848,19 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>295</v>
+        <v>339</v>
       </c>
       <c r="B10" t="s">
-        <v>300</v>
+        <v>361</v>
       </c>
       <c r="C10" t="s">
-        <v>299</v>
+        <v>362</v>
       </c>
       <c r="D10" t="s">
-        <v>298</v>
+        <v>360</v>
       </c>
       <c r="E10">
-        <v>1996</v>
+        <v>1999</v>
       </c>
       <c r="F10" t="s">
         <v>290</v>
@@ -1631,19 +1871,19 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>293</v>
+        <v>340</v>
       </c>
       <c r="B11" t="s">
-        <v>296</v>
+        <v>358</v>
       </c>
       <c r="C11" t="s">
-        <v>304</v>
+        <v>359</v>
       </c>
       <c r="D11" t="s">
-        <v>303</v>
+        <v>360</v>
       </c>
       <c r="E11">
-        <v>2000</v>
+        <v>1999</v>
       </c>
       <c r="F11" t="s">
         <v>290</v>
@@ -1654,19 +1894,19 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>292</v>
+        <v>341</v>
       </c>
       <c r="B12" t="s">
-        <v>296</v>
+        <v>356</v>
       </c>
       <c r="C12" t="s">
-        <v>297</v>
+        <v>357</v>
       </c>
       <c r="D12" t="s">
-        <v>303</v>
+        <v>355</v>
       </c>
       <c r="E12">
-        <v>1999</v>
+        <v>2001</v>
       </c>
       <c r="F12" t="s">
         <v>290</v>
@@ -1677,19 +1917,19 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>288</v>
+        <v>342</v>
       </c>
       <c r="B13" t="s">
-        <v>3</v>
+        <v>353</v>
       </c>
       <c r="C13" t="s">
-        <v>286</v>
+        <v>354</v>
       </c>
       <c r="D13" t="s">
-        <v>287</v>
+        <v>355</v>
       </c>
       <c r="E13">
-        <v>1999</v>
+        <v>2001</v>
       </c>
       <c r="F13" t="s">
         <v>290</v>
@@ -1700,22 +1940,22 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>289</v>
+        <v>343</v>
       </c>
       <c r="B14" t="s">
-        <v>284</v>
+        <v>3</v>
       </c>
       <c r="C14" t="s">
-        <v>285</v>
+        <v>352</v>
       </c>
       <c r="D14" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="E14">
-        <v>1993</v>
+        <v>1999</v>
       </c>
       <c r="F14" t="s">
-        <v>290</v>
+        <v>379</v>
       </c>
       <c r="G14" t="s">
         <v>241</v>
@@ -1723,16 +1963,16 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>231</v>
+        <v>344</v>
       </c>
       <c r="B15" t="s">
-        <v>229</v>
+        <v>349</v>
       </c>
       <c r="C15" t="s">
-        <v>229</v>
+        <v>350</v>
       </c>
       <c r="D15" t="s">
-        <v>230</v>
+        <v>351</v>
       </c>
       <c r="E15">
         <v>1996</v>
@@ -1746,19 +1986,19 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>234</v>
+        <v>324</v>
       </c>
       <c r="B16" t="s">
-        <v>227</v>
+        <v>325</v>
       </c>
       <c r="C16" t="s">
-        <v>227</v>
+        <v>326</v>
       </c>
       <c r="D16" t="s">
-        <v>228</v>
+        <v>327</v>
       </c>
       <c r="E16">
-        <v>1998</v>
+        <v>2002</v>
       </c>
       <c r="F16" t="s">
         <v>290</v>
@@ -1769,19 +2009,19 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>232</v>
+        <v>323</v>
       </c>
       <c r="B17" t="s">
-        <v>224</v>
+        <v>3</v>
       </c>
       <c r="C17" t="s">
-        <v>222</v>
+        <v>328</v>
       </c>
       <c r="D17" t="s">
-        <v>223</v>
+        <v>329</v>
       </c>
       <c r="E17">
-        <v>2005</v>
+        <v>1995</v>
       </c>
       <c r="F17" t="s">
         <v>290</v>
@@ -1792,19 +2032,19 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>233</v>
+        <v>319</v>
       </c>
       <c r="B18" t="s">
-        <v>221</v>
+        <v>321</v>
       </c>
       <c r="C18" t="s">
-        <v>226</v>
+        <v>322</v>
       </c>
       <c r="D18" t="s">
-        <v>225</v>
+        <v>173</v>
       </c>
       <c r="E18">
-        <v>1997</v>
+        <v>1995</v>
       </c>
       <c r="F18" t="s">
         <v>290</v>
@@ -1815,19 +2055,19 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>157</v>
+        <v>318</v>
       </c>
       <c r="B19" t="s">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="C19" t="s">
-        <v>105</v>
+        <v>320</v>
       </c>
       <c r="D19" t="s">
         <v>173</v>
       </c>
       <c r="E19">
-        <v>1998</v>
+        <v>2001</v>
       </c>
       <c r="F19" t="s">
         <v>290</v>
@@ -1838,19 +2078,19 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>108</v>
+        <v>306</v>
       </c>
       <c r="B20" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C20" t="s">
-        <v>1</v>
+        <v>309</v>
       </c>
       <c r="D20" t="s">
-        <v>2</v>
+        <v>310</v>
       </c>
       <c r="E20">
-        <v>1995</v>
+        <v>1997</v>
       </c>
       <c r="F20" t="s">
         <v>290</v>
@@ -1861,16 +2101,16 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>118</v>
+        <v>307</v>
       </c>
       <c r="B21" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C21" t="s">
-        <v>281</v>
+        <v>311</v>
       </c>
       <c r="D21" t="s">
-        <v>170</v>
+        <v>312</v>
       </c>
       <c r="E21">
         <v>1998</v>
@@ -1884,16 +2124,16 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>109</v>
+        <v>308</v>
       </c>
       <c r="B22" t="s">
-        <v>3</v>
+        <v>313</v>
       </c>
       <c r="C22" t="s">
-        <v>4</v>
+        <v>314</v>
       </c>
       <c r="D22" t="s">
-        <v>2</v>
+        <v>171</v>
       </c>
       <c r="E22">
         <v>1996</v>
@@ -1907,19 +2147,19 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>119</v>
+        <v>305</v>
       </c>
       <c r="B23" t="s">
-        <v>3</v>
+        <v>315</v>
       </c>
       <c r="C23" t="s">
-        <v>54</v>
+        <v>316</v>
       </c>
       <c r="D23" t="s">
-        <v>171</v>
+        <v>317</v>
       </c>
       <c r="E23">
-        <v>1999</v>
+        <v>1996</v>
       </c>
       <c r="F23" t="s">
         <v>290</v>
@@ -1930,19 +2170,19 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>129</v>
+        <v>294</v>
       </c>
       <c r="B24" t="s">
-        <v>3</v>
+        <v>301</v>
       </c>
       <c r="C24" t="s">
-        <v>59</v>
+        <v>302</v>
       </c>
       <c r="D24" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E24">
-        <v>2003</v>
+        <v>1999</v>
       </c>
       <c r="F24" t="s">
         <v>290</v>
@@ -1953,16 +2193,16 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>110</v>
+        <v>295</v>
       </c>
       <c r="B25" t="s">
-        <v>5</v>
+        <v>300</v>
       </c>
       <c r="C25" t="s">
-        <v>46</v>
+        <v>299</v>
       </c>
       <c r="D25" t="s">
-        <v>202</v>
+        <v>298</v>
       </c>
       <c r="E25">
         <v>1996</v>
@@ -1976,19 +2216,19 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>126</v>
+        <v>293</v>
       </c>
       <c r="B26" t="s">
-        <v>5</v>
+        <v>296</v>
       </c>
       <c r="C26" t="s">
-        <v>63</v>
+        <v>304</v>
       </c>
       <c r="D26" t="s">
-        <v>175</v>
+        <v>303</v>
       </c>
       <c r="E26">
-        <v>2015</v>
+        <v>2000</v>
       </c>
       <c r="F26" t="s">
         <v>290</v>
@@ -1999,42 +2239,42 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>135</v>
+        <v>292</v>
       </c>
       <c r="B27" t="s">
-        <v>5</v>
+        <v>296</v>
       </c>
       <c r="C27" t="s">
-        <v>93</v>
+        <v>297</v>
       </c>
       <c r="D27" t="s">
-        <v>202</v>
+        <v>303</v>
       </c>
       <c r="E27">
-        <v>2024</v>
+        <v>1999</v>
       </c>
       <c r="F27" t="s">
         <v>290</v>
       </c>
       <c r="G27" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>111</v>
+        <v>345</v>
       </c>
       <c r="B28" t="s">
-        <v>6</v>
+        <v>346</v>
       </c>
       <c r="C28" t="s">
-        <v>47</v>
+        <v>347</v>
       </c>
       <c r="D28" t="s">
-        <v>165</v>
+        <v>348</v>
       </c>
       <c r="E28">
-        <v>1996</v>
+        <v>1997</v>
       </c>
       <c r="F28" t="s">
         <v>290</v>
@@ -2045,19 +2285,19 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>220</v>
+        <v>288</v>
       </c>
       <c r="B29" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C29" t="s">
-        <v>219</v>
+        <v>286</v>
       </c>
       <c r="D29" t="s">
-        <v>166</v>
+        <v>287</v>
       </c>
       <c r="E29">
-        <v>1997</v>
+        <v>1999</v>
       </c>
       <c r="F29" t="s">
         <v>290</v>
@@ -2068,19 +2308,19 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>112</v>
+        <v>289</v>
       </c>
       <c r="B30" t="s">
-        <v>7</v>
+        <v>284</v>
       </c>
       <c r="C30" t="s">
-        <v>48</v>
+        <v>285</v>
       </c>
       <c r="D30" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="E30">
-        <v>1997</v>
+        <v>1993</v>
       </c>
       <c r="F30" t="s">
         <v>290</v>
@@ -2091,19 +2331,19 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>113</v>
+        <v>231</v>
       </c>
       <c r="B31" t="s">
-        <v>7</v>
+        <v>229</v>
       </c>
       <c r="C31" t="s">
-        <v>49</v>
+        <v>229</v>
       </c>
       <c r="D31" t="s">
-        <v>166</v>
+        <v>230</v>
       </c>
       <c r="E31">
-        <v>1997</v>
+        <v>1996</v>
       </c>
       <c r="F31" t="s">
         <v>290</v>
@@ -2114,19 +2354,19 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>120</v>
+        <v>234</v>
       </c>
       <c r="B32" t="s">
-        <v>7</v>
+        <v>227</v>
       </c>
       <c r="C32" t="s">
-        <v>55</v>
+        <v>227</v>
       </c>
       <c r="D32" t="s">
-        <v>166</v>
+        <v>228</v>
       </c>
       <c r="E32">
-        <v>2000</v>
+        <v>1998</v>
       </c>
       <c r="F32" t="s">
         <v>290</v>
@@ -2137,19 +2377,19 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>122</v>
+        <v>232</v>
       </c>
       <c r="B33" t="s">
-        <v>7</v>
+        <v>224</v>
       </c>
       <c r="C33" t="s">
-        <v>57</v>
+        <v>222</v>
       </c>
       <c r="D33" t="s">
-        <v>166</v>
+        <v>223</v>
       </c>
       <c r="E33">
-        <v>2002</v>
+        <v>2005</v>
       </c>
       <c r="F33" t="s">
         <v>290</v>
@@ -2160,16 +2400,16 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>114</v>
+        <v>233</v>
       </c>
       <c r="B34" t="s">
-        <v>8</v>
+        <v>221</v>
       </c>
       <c r="C34" t="s">
-        <v>50</v>
+        <v>226</v>
       </c>
       <c r="D34" t="s">
-        <v>167</v>
+        <v>225</v>
       </c>
       <c r="E34">
         <v>1997</v>
@@ -2183,19 +2423,19 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>115</v>
+        <v>157</v>
       </c>
       <c r="B35" t="s">
-        <v>9</v>
+        <v>45</v>
       </c>
       <c r="C35" t="s">
-        <v>51</v>
+        <v>105</v>
       </c>
       <c r="D35" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="E35">
-        <v>1997</v>
+        <v>1998</v>
       </c>
       <c r="F35" t="s">
         <v>290</v>
@@ -2206,19 +2446,19 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="B36" t="s">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C36" t="s">
-        <v>52</v>
+        <v>1</v>
       </c>
       <c r="D36" t="s">
-        <v>168</v>
+        <v>2</v>
       </c>
       <c r="E36">
-        <v>1997</v>
+        <v>1995</v>
       </c>
       <c r="F36" t="s">
         <v>290</v>
@@ -2229,19 +2469,19 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B37" t="s">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="C37" t="s">
-        <v>53</v>
+        <v>281</v>
       </c>
       <c r="D37" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E37">
-        <v>1997</v>
+        <v>1998</v>
       </c>
       <c r="F37" t="s">
         <v>290</v>
@@ -2252,22 +2492,22 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="B38" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="C38" t="s">
-        <v>56</v>
+        <v>4</v>
       </c>
       <c r="D38" t="s">
-        <v>172</v>
+        <v>2</v>
       </c>
       <c r="E38">
-        <v>2001</v>
+        <v>1996</v>
       </c>
       <c r="F38" t="s">
-        <v>235</v>
+        <v>290</v>
       </c>
       <c r="G38" t="s">
         <v>241</v>
@@ -2275,19 +2515,19 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>132</v>
+        <v>119</v>
       </c>
       <c r="B39" t="s">
-        <v>301</v>
+        <v>3</v>
       </c>
       <c r="C39" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="D39" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E39">
-        <v>2002</v>
+        <v>1999</v>
       </c>
       <c r="F39" t="s">
         <v>290</v>
@@ -2298,22 +2538,22 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>209</v>
+        <v>129</v>
       </c>
       <c r="B40" t="s">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="C40" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="D40" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="E40">
         <v>2003</v>
       </c>
       <c r="F40" t="s">
-        <v>235</v>
+        <v>290</v>
       </c>
       <c r="G40" t="s">
         <v>241</v>
@@ -2321,22 +2561,22 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>123</v>
+        <v>110</v>
       </c>
       <c r="B41" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C41" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="D41" t="s">
-        <v>174</v>
+        <v>202</v>
       </c>
       <c r="E41">
-        <v>2004</v>
+        <v>1996</v>
       </c>
       <c r="F41" t="s">
-        <v>235</v>
+        <v>290</v>
       </c>
       <c r="G41" t="s">
         <v>241</v>
@@ -2344,22 +2584,22 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B42" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C42" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D42" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E42">
-        <v>2004</v>
+        <v>2015</v>
       </c>
       <c r="F42" t="s">
-        <v>235</v>
+        <v>290</v>
       </c>
       <c r="G42" t="s">
         <v>241</v>
@@ -2367,42 +2607,42 @@
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="B43" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="C43" t="s">
-        <v>62</v>
+        <v>93</v>
       </c>
       <c r="D43" t="s">
-        <v>174</v>
+        <v>202</v>
       </c>
       <c r="E43">
-        <v>2004</v>
+        <v>2024</v>
       </c>
       <c r="F43" t="s">
-        <v>235</v>
+        <v>290</v>
       </c>
       <c r="G43" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="B44" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="C44" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="D44" t="s">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="E44">
-        <v>2017</v>
+        <v>1996</v>
       </c>
       <c r="F44" t="s">
         <v>290</v>
@@ -2413,19 +2653,19 @@
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>137</v>
+        <v>220</v>
       </c>
       <c r="B45" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="C45" t="s">
-        <v>65</v>
+        <v>219</v>
       </c>
       <c r="D45" t="s">
-        <v>177</v>
+        <v>166</v>
       </c>
       <c r="E45">
-        <v>1999</v>
+        <v>1997</v>
       </c>
       <c r="F45" t="s">
         <v>290</v>
@@ -2436,19 +2676,19 @@
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>134</v>
+        <v>112</v>
       </c>
       <c r="B46" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C46" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="D46" t="s">
-        <v>178</v>
+        <v>166</v>
       </c>
       <c r="E46">
-        <v>2025</v>
+        <v>1997</v>
       </c>
       <c r="F46" t="s">
         <v>290</v>
@@ -2459,42 +2699,42 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>131</v>
+        <v>113</v>
       </c>
       <c r="B47" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="C47" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D47" t="s">
-        <v>179</v>
+        <v>166</v>
       </c>
       <c r="E47">
-        <v>2024</v>
+        <v>1997</v>
       </c>
       <c r="F47" t="s">
         <v>290</v>
       </c>
       <c r="G47" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>133</v>
+        <v>120</v>
       </c>
       <c r="B48" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C48" t="s">
-        <v>69</v>
+        <v>55</v>
       </c>
       <c r="D48" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="E48">
-        <v>2023</v>
+        <v>2000</v>
       </c>
       <c r="F48" t="s">
         <v>290</v>
@@ -2505,22 +2745,22 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>148</v>
+        <v>122</v>
       </c>
       <c r="B49" t="s">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="C49" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="D49" t="s">
-        <v>181</v>
+        <v>166</v>
       </c>
       <c r="E49">
-        <v>1991</v>
+        <v>2002</v>
       </c>
       <c r="F49" t="s">
-        <v>235</v>
+        <v>290</v>
       </c>
       <c r="G49" t="s">
         <v>241</v>
@@ -2528,22 +2768,22 @@
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>149</v>
+        <v>114</v>
       </c>
       <c r="B50" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="C50" t="s">
-        <v>71</v>
+        <v>50</v>
       </c>
       <c r="D50" t="s">
-        <v>181</v>
+        <v>167</v>
       </c>
       <c r="E50">
-        <v>1993</v>
+        <v>1997</v>
       </c>
       <c r="F50" t="s">
-        <v>235</v>
+        <v>290</v>
       </c>
       <c r="G50" t="s">
         <v>241</v>
@@ -2551,22 +2791,22 @@
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>153</v>
+        <v>115</v>
       </c>
       <c r="B51" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="C51" t="s">
-        <v>95</v>
+        <v>51</v>
       </c>
       <c r="D51" t="s">
-        <v>181</v>
+        <v>168</v>
       </c>
       <c r="E51">
-        <v>2003</v>
+        <v>1997</v>
       </c>
       <c r="F51" t="s">
-        <v>235</v>
+        <v>290</v>
       </c>
       <c r="G51" t="s">
         <v>241</v>
@@ -2574,22 +2814,22 @@
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>130</v>
+        <v>116</v>
       </c>
       <c r="B52" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="C52" t="s">
-        <v>94</v>
+        <v>52</v>
       </c>
       <c r="D52" t="s">
-        <v>182</v>
+        <v>168</v>
       </c>
       <c r="E52">
-        <v>2016</v>
+        <v>1997</v>
       </c>
       <c r="F52" t="s">
-        <v>235</v>
+        <v>290</v>
       </c>
       <c r="G52" t="s">
         <v>241</v>
@@ -2597,22 +2837,22 @@
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>155</v>
+        <v>117</v>
       </c>
       <c r="B53" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="C53" t="s">
-        <v>72</v>
+        <v>53</v>
       </c>
       <c r="D53" t="s">
-        <v>183</v>
+        <v>169</v>
       </c>
       <c r="E53">
-        <v>2000</v>
+        <v>1997</v>
       </c>
       <c r="F53" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G53" t="s">
         <v>241</v>
@@ -2620,19 +2860,19 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>146</v>
+        <v>121</v>
       </c>
       <c r="B54" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="C54" t="s">
-        <v>73</v>
+        <v>56</v>
       </c>
       <c r="D54" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="E54">
-        <v>2005</v>
+        <v>2001</v>
       </c>
       <c r="F54" t="s">
         <v>235</v>
@@ -2643,22 +2883,22 @@
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="B55" t="s">
-        <v>24</v>
+        <v>301</v>
       </c>
       <c r="C55" t="s">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="D55" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="E55">
-        <v>1993</v>
+        <v>2002</v>
       </c>
       <c r="F55" t="s">
-        <v>235</v>
+        <v>290</v>
       </c>
       <c r="G55" t="s">
         <v>241</v>
@@ -2666,19 +2906,19 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>245</v>
+        <v>209</v>
       </c>
       <c r="B56" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="C56" t="s">
-        <v>246</v>
+        <v>68</v>
       </c>
       <c r="D56" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="E56">
-        <v>2000</v>
+        <v>2003</v>
       </c>
       <c r="F56" t="s">
         <v>235</v>
@@ -2689,19 +2929,19 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>145</v>
+        <v>123</v>
       </c>
       <c r="B57" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="C57" t="s">
-        <v>164</v>
+        <v>60</v>
       </c>
       <c r="D57" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="E57">
-        <v>1995</v>
+        <v>2004</v>
       </c>
       <c r="F57" t="s">
         <v>235</v>
@@ -2712,19 +2952,19 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>277</v>
+        <v>124</v>
       </c>
       <c r="B58" t="s">
-        <v>278</v>
+        <v>13</v>
       </c>
       <c r="C58" t="s">
-        <v>279</v>
+        <v>61</v>
       </c>
       <c r="D58" t="s">
-        <v>280</v>
+        <v>174</v>
       </c>
       <c r="E58">
-        <v>2003</v>
+        <v>2004</v>
       </c>
       <c r="F58" t="s">
         <v>235</v>
@@ -2735,16 +2975,16 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>158</v>
+        <v>125</v>
       </c>
       <c r="B59" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="C59" t="s">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="D59" t="s">
-        <v>187</v>
+        <v>174</v>
       </c>
       <c r="E59">
         <v>2004</v>
@@ -2758,22 +2998,22 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>152</v>
+        <v>127</v>
       </c>
       <c r="B60" t="s">
-        <v>78</v>
+        <v>15</v>
       </c>
       <c r="C60" t="s">
-        <v>79</v>
+        <v>64</v>
       </c>
       <c r="D60" t="s">
-        <v>190</v>
+        <v>176</v>
       </c>
       <c r="E60">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="F60" t="s">
-        <v>235</v>
+        <v>290</v>
       </c>
       <c r="G60" t="s">
         <v>241</v>
@@ -2781,19 +3021,19 @@
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>210</v>
+        <v>137</v>
       </c>
       <c r="B61" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="C61" t="s">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="D61" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
       <c r="E61">
-        <v>2003</v>
+        <v>1999</v>
       </c>
       <c r="F61" t="s">
         <v>290</v>
@@ -2804,22 +3044,22 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B62" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="C62" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="D62" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
       <c r="E62">
-        <v>2020</v>
+        <v>2025</v>
       </c>
       <c r="F62" t="s">
-        <v>235</v>
+        <v>290</v>
       </c>
       <c r="G62" t="s">
         <v>241</v>
@@ -2827,45 +3067,45 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>211</v>
+        <v>131</v>
       </c>
       <c r="B63" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="C63" t="s">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="D63" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="E63">
-        <v>1995</v>
+        <v>2024</v>
       </c>
       <c r="F63" t="s">
-        <v>235</v>
+        <v>290</v>
       </c>
       <c r="G63" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>161</v>
+        <v>133</v>
       </c>
       <c r="B64" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="C64" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="D64" t="s">
-        <v>192</v>
+        <v>173</v>
       </c>
       <c r="E64">
-        <v>1996</v>
+        <v>2023</v>
       </c>
       <c r="F64" t="s">
-        <v>235</v>
+        <v>290</v>
       </c>
       <c r="G64" t="s">
         <v>241</v>
@@ -2873,22 +3113,22 @@
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="B65" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="C65" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="D65" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="E65">
-        <v>1976</v>
+        <v>1991</v>
       </c>
       <c r="F65" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="G65" t="s">
         <v>241</v>
@@ -2896,45 +3136,45 @@
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>274</v>
+        <v>149</v>
       </c>
       <c r="B66" t="s">
-        <v>272</v>
+        <v>21</v>
       </c>
       <c r="C66" t="s">
-        <v>273</v>
+        <v>71</v>
       </c>
       <c r="D66" t="s">
-        <v>275</v>
+        <v>181</v>
       </c>
       <c r="E66">
-        <v>2025</v>
+        <v>1993</v>
       </c>
       <c r="F66" t="s">
-        <v>290</v>
+        <v>235</v>
       </c>
       <c r="G66" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>128</v>
+        <v>153</v>
       </c>
       <c r="B67" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="C67" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="D67" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="E67">
-        <v>1961</v>
+        <v>2003</v>
       </c>
       <c r="F67" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="G67" t="s">
         <v>241</v>
@@ -2942,22 +3182,22 @@
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="B68" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="C68" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="D68" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="E68">
-        <v>2018</v>
+        <v>2016</v>
       </c>
       <c r="F68" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="G68" t="s">
         <v>241</v>
@@ -2965,42 +3205,42 @@
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="B69" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="C69" t="s">
-        <v>85</v>
+        <v>72</v>
       </c>
       <c r="D69" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="E69">
-        <v>2017</v>
+        <v>2000</v>
       </c>
       <c r="F69" t="s">
-        <v>239</v>
+        <v>291</v>
       </c>
       <c r="G69" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>163</v>
+        <v>146</v>
       </c>
       <c r="B70" t="s">
-        <v>237</v>
+        <v>23</v>
       </c>
       <c r="C70" t="s">
-        <v>86</v>
+        <v>73</v>
       </c>
       <c r="D70" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="E70">
-        <v>2007</v>
+        <v>2005</v>
       </c>
       <c r="F70" t="s">
         <v>235</v>
@@ -3011,22 +3251,22 @@
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="B71" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="C71" t="s">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="D71" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="E71">
-        <v>2014</v>
+        <v>1993</v>
       </c>
       <c r="F71" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="G71" t="s">
         <v>241</v>
@@ -3034,22 +3274,22 @@
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>154</v>
+        <v>245</v>
       </c>
       <c r="B72" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="C72" t="s">
-        <v>88</v>
+        <v>246</v>
       </c>
       <c r="D72" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
       <c r="E72">
-        <v>2016</v>
+        <v>2000</v>
       </c>
       <c r="F72" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="G72" t="s">
         <v>241</v>
@@ -3057,22 +3297,22 @@
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>159</v>
+        <v>145</v>
       </c>
       <c r="B73" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="C73" t="s">
-        <v>89</v>
+        <v>164</v>
       </c>
       <c r="D73" t="s">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="E73">
-        <v>2010</v>
+        <v>1995</v>
       </c>
       <c r="F73" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="G73" t="s">
         <v>241</v>
@@ -3080,45 +3320,45 @@
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>160</v>
+        <v>277</v>
       </c>
       <c r="B74" t="s">
-        <v>35</v>
+        <v>278</v>
       </c>
       <c r="C74" t="s">
-        <v>90</v>
+        <v>279</v>
       </c>
       <c r="D74" t="s">
-        <v>198</v>
+        <v>280</v>
       </c>
       <c r="E74">
-        <v>2012</v>
+        <v>2003</v>
       </c>
       <c r="F74" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="G74" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="B75" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="C75" t="s">
-        <v>283</v>
+        <v>75</v>
       </c>
       <c r="D75" t="s">
-        <v>200</v>
+        <v>187</v>
       </c>
       <c r="E75">
-        <v>1995</v>
+        <v>2004</v>
       </c>
       <c r="F75" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="G75" t="s">
         <v>241</v>
@@ -3126,160 +3366,160 @@
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>141</v>
+        <v>152</v>
       </c>
       <c r="B76" t="s">
-        <v>37</v>
+        <v>78</v>
       </c>
       <c r="C76" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="D76" t="s">
-        <v>199</v>
+        <v>190</v>
       </c>
       <c r="E76">
-        <v>1971</v>
+        <v>2016</v>
       </c>
       <c r="F76" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="G76" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>147</v>
+        <v>210</v>
       </c>
       <c r="B77" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="C77" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="D77" t="s">
-        <v>201</v>
+        <v>188</v>
       </c>
       <c r="E77">
-        <v>1982</v>
+        <v>2003</v>
       </c>
       <c r="F77" t="s">
-        <v>236</v>
+        <v>290</v>
       </c>
       <c r="G77" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B78" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="C78" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="D78" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="E78">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="F78" t="s">
-        <v>290</v>
+        <v>235</v>
       </c>
       <c r="G78" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B79" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="C79" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="D79" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="E79">
-        <v>1977</v>
+        <v>1995</v>
       </c>
       <c r="F79" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="G79" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>214</v>
+        <v>161</v>
       </c>
       <c r="B80" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="C80" t="s">
-        <v>99</v>
+        <v>81</v>
       </c>
       <c r="D80" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="E80">
-        <v>1978</v>
+        <v>1996</v>
       </c>
       <c r="F80" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="G80" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="B81" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="C81" t="s">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="D81" t="s">
-        <v>204</v>
+        <v>186</v>
       </c>
       <c r="E81">
-        <v>1980</v>
+        <v>1976</v>
       </c>
       <c r="F81" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="G81" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>215</v>
+        <v>274</v>
       </c>
       <c r="B82" t="s">
-        <v>43</v>
+        <v>272</v>
       </c>
       <c r="C82" t="s">
-        <v>43</v>
+        <v>273</v>
       </c>
       <c r="D82" t="s">
-        <v>205</v>
+        <v>275</v>
       </c>
       <c r="E82">
-        <v>1978</v>
+        <v>2025</v>
       </c>
       <c r="F82" t="s">
-        <v>236</v>
+        <v>290</v>
       </c>
       <c r="G82" t="s">
         <v>243</v>
@@ -3287,68 +3527,68 @@
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>218</v>
+        <v>128</v>
       </c>
       <c r="B83" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="C83" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="D83" t="s">
-        <v>205</v>
+        <v>193</v>
       </c>
       <c r="E83">
-        <v>1979</v>
+        <v>1961</v>
       </c>
       <c r="F83" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G83" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B84" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="C84" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
       <c r="D84" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="E84">
-        <v>1985</v>
+        <v>2018</v>
       </c>
       <c r="F84" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G84" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>216</v>
+        <v>162</v>
       </c>
       <c r="B85" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="C85" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="D85" t="s">
-        <v>207</v>
+        <v>194</v>
       </c>
       <c r="E85">
-        <v>1985</v>
+        <v>2017</v>
       </c>
       <c r="F85" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G85" t="s">
         <v>243</v>
@@ -3356,42 +3596,42 @@
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>217</v>
+        <v>163</v>
       </c>
       <c r="B86" t="s">
-        <v>44</v>
+        <v>237</v>
       </c>
       <c r="C86" t="s">
-        <v>104</v>
+        <v>86</v>
       </c>
       <c r="D86" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="E86">
-        <v>1971</v>
+        <v>2007</v>
       </c>
       <c r="F86" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="G86" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B87" t="s">
-        <v>106</v>
+        <v>33</v>
       </c>
       <c r="C87" t="s">
-        <v>107</v>
+        <v>87</v>
       </c>
       <c r="D87" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="E87">
-        <v>2017</v>
+        <v>2014</v>
       </c>
       <c r="F87" t="s">
         <v>239</v>
@@ -3402,22 +3642,22 @@
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>262</v>
+        <v>154</v>
       </c>
       <c r="B88" t="s">
-        <v>247</v>
+        <v>34</v>
       </c>
       <c r="C88" t="s">
-        <v>250</v>
+        <v>88</v>
       </c>
       <c r="D88" t="s">
-        <v>256</v>
+        <v>197</v>
       </c>
       <c r="E88">
-        <v>2010</v>
+        <v>2016</v>
       </c>
       <c r="F88" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="G88" t="s">
         <v>241</v>
@@ -3425,22 +3665,22 @@
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>276</v>
+        <v>159</v>
       </c>
       <c r="B89" t="s">
-        <v>247</v>
+        <v>35</v>
       </c>
       <c r="C89" t="s">
-        <v>248</v>
+        <v>89</v>
       </c>
       <c r="D89" t="s">
-        <v>257</v>
+        <v>198</v>
       </c>
       <c r="E89">
-        <v>2011</v>
+        <v>2010</v>
       </c>
       <c r="F89" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="G89" t="s">
         <v>241</v>
@@ -3448,45 +3688,45 @@
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>263</v>
+        <v>160</v>
       </c>
       <c r="B90" t="s">
-        <v>247</v>
+        <v>35</v>
       </c>
       <c r="C90" t="s">
-        <v>249</v>
+        <v>90</v>
       </c>
       <c r="D90" t="s">
-        <v>258</v>
+        <v>198</v>
       </c>
       <c r="E90">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="F90" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="G90" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>264</v>
+        <v>150</v>
       </c>
       <c r="B91" t="s">
-        <v>247</v>
+        <v>36</v>
       </c>
       <c r="C91" t="s">
-        <v>252</v>
+        <v>283</v>
       </c>
       <c r="D91" t="s">
-        <v>258</v>
+        <v>200</v>
       </c>
       <c r="E91">
-        <v>2015</v>
+        <v>1995</v>
       </c>
       <c r="F91" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="G91" t="s">
         <v>241</v>
@@ -3494,91 +3734,91 @@
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>265</v>
+        <v>141</v>
       </c>
       <c r="B92" t="s">
-        <v>247</v>
+        <v>37</v>
       </c>
       <c r="C92" t="s">
-        <v>251</v>
+        <v>91</v>
       </c>
       <c r="D92" t="s">
-        <v>186</v>
+        <v>199</v>
       </c>
       <c r="E92">
-        <v>2017</v>
+        <v>1971</v>
       </c>
       <c r="F92" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="G92" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>266</v>
+        <v>147</v>
       </c>
       <c r="B93" t="s">
-        <v>253</v>
+        <v>38</v>
       </c>
       <c r="C93" t="s">
-        <v>254</v>
+        <v>92</v>
       </c>
       <c r="D93" t="s">
-        <v>186</v>
+        <v>201</v>
       </c>
       <c r="E93">
-        <v>2013</v>
+        <v>1982</v>
       </c>
       <c r="F93" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="G93" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>267</v>
+        <v>138</v>
       </c>
       <c r="B94" t="s">
-        <v>253</v>
+        <v>39</v>
       </c>
       <c r="C94" t="s">
-        <v>255</v>
+        <v>96</v>
       </c>
       <c r="D94" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="E94">
-        <v>2015</v>
+        <v>2021</v>
       </c>
       <c r="F94" t="s">
-        <v>235</v>
+        <v>290</v>
       </c>
       <c r="G94" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>268</v>
+        <v>213</v>
       </c>
       <c r="B95" t="s">
-        <v>260</v>
+        <v>41</v>
       </c>
       <c r="C95" t="s">
-        <v>259</v>
+        <v>98</v>
       </c>
       <c r="D95" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E95">
-        <v>1982</v>
+        <v>1977</v>
       </c>
       <c r="F95" t="s">
-        <v>261</v>
+        <v>238</v>
       </c>
       <c r="G95" t="s">
         <v>243</v>
@@ -3586,22 +3826,22 @@
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
       <c r="B96" t="s">
-        <v>3</v>
+        <v>41</v>
       </c>
       <c r="C96" t="s">
-        <v>270</v>
+        <v>99</v>
       </c>
       <c r="D96" t="s">
-        <v>271</v>
+        <v>203</v>
       </c>
       <c r="E96">
-        <v>2018</v>
+        <v>1978</v>
       </c>
       <c r="F96" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="G96" t="s">
         <v>243</v>
@@ -3609,36 +3849,419 @@
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>212</v>
+        <v>156</v>
       </c>
       <c r="B97" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C97" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D97" t="s">
-        <v>282</v>
+        <v>204</v>
       </c>
       <c r="E97">
-        <v>1962</v>
+        <v>1980</v>
       </c>
       <c r="F97" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="G97" t="s">
         <v>243</v>
       </c>
     </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
+        <v>215</v>
+      </c>
+      <c r="B98" t="s">
+        <v>43</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98" t="s">
+        <v>205</v>
+      </c>
+      <c r="E98">
+        <v>1978</v>
+      </c>
+      <c r="F98" t="s">
+        <v>236</v>
+      </c>
+      <c r="G98" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A99" t="s">
+        <v>218</v>
+      </c>
+      <c r="B99" t="s">
+        <v>43</v>
+      </c>
+      <c r="C99" t="s">
+        <v>101</v>
+      </c>
+      <c r="D99" t="s">
+        <v>205</v>
+      </c>
+      <c r="E99">
+        <v>1979</v>
+      </c>
+      <c r="F99" t="s">
+        <v>236</v>
+      </c>
+      <c r="G99" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A100" t="s">
+        <v>142</v>
+      </c>
+      <c r="B100" t="s">
+        <v>43</v>
+      </c>
+      <c r="C100" t="s">
+        <v>102</v>
+      </c>
+      <c r="D100" t="s">
+        <v>206</v>
+      </c>
+      <c r="E100">
+        <v>1985</v>
+      </c>
+      <c r="F100" t="s">
+        <v>236</v>
+      </c>
+      <c r="G100" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A101" t="s">
+        <v>216</v>
+      </c>
+      <c r="B101" t="s">
+        <v>44</v>
+      </c>
+      <c r="C101" t="s">
+        <v>103</v>
+      </c>
+      <c r="D101" t="s">
+        <v>207</v>
+      </c>
+      <c r="E101">
+        <v>1985</v>
+      </c>
+      <c r="F101" t="s">
+        <v>236</v>
+      </c>
+      <c r="G101" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A102" t="s">
+        <v>217</v>
+      </c>
+      <c r="B102" t="s">
+        <v>44</v>
+      </c>
+      <c r="C102" t="s">
+        <v>104</v>
+      </c>
+      <c r="D102" t="s">
+        <v>203</v>
+      </c>
+      <c r="E102">
+        <v>1971</v>
+      </c>
+      <c r="F102" t="s">
+        <v>236</v>
+      </c>
+      <c r="G102" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A103" t="s">
+        <v>139</v>
+      </c>
+      <c r="B103" t="s">
+        <v>106</v>
+      </c>
+      <c r="C103" t="s">
+        <v>107</v>
+      </c>
+      <c r="D103" t="s">
+        <v>208</v>
+      </c>
+      <c r="E103">
+        <v>2017</v>
+      </c>
+      <c r="F103" t="s">
+        <v>239</v>
+      </c>
+      <c r="G103" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A104" t="s">
+        <v>262</v>
+      </c>
+      <c r="B104" t="s">
+        <v>247</v>
+      </c>
+      <c r="C104" t="s">
+        <v>250</v>
+      </c>
+      <c r="D104" t="s">
+        <v>256</v>
+      </c>
+      <c r="E104">
+        <v>2010</v>
+      </c>
+      <c r="F104" t="s">
+        <v>235</v>
+      </c>
+      <c r="G104" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A105" t="s">
+        <v>276</v>
+      </c>
+      <c r="B105" t="s">
+        <v>247</v>
+      </c>
+      <c r="C105" t="s">
+        <v>248</v>
+      </c>
+      <c r="D105" t="s">
+        <v>257</v>
+      </c>
+      <c r="E105">
+        <v>2011</v>
+      </c>
+      <c r="F105" t="s">
+        <v>235</v>
+      </c>
+      <c r="G105" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A106" t="s">
+        <v>263</v>
+      </c>
+      <c r="B106" t="s">
+        <v>247</v>
+      </c>
+      <c r="C106" t="s">
+        <v>249</v>
+      </c>
+      <c r="D106" t="s">
+        <v>258</v>
+      </c>
+      <c r="E106">
+        <v>2013</v>
+      </c>
+      <c r="F106" t="s">
+        <v>235</v>
+      </c>
+      <c r="G106" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A107" t="s">
+        <v>264</v>
+      </c>
+      <c r="B107" t="s">
+        <v>247</v>
+      </c>
+      <c r="C107" t="s">
+        <v>252</v>
+      </c>
+      <c r="D107" t="s">
+        <v>258</v>
+      </c>
+      <c r="E107">
+        <v>2015</v>
+      </c>
+      <c r="F107" t="s">
+        <v>235</v>
+      </c>
+      <c r="G107" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A108" t="s">
+        <v>265</v>
+      </c>
+      <c r="B108" t="s">
+        <v>247</v>
+      </c>
+      <c r="C108" t="s">
+        <v>251</v>
+      </c>
+      <c r="D108" t="s">
+        <v>186</v>
+      </c>
+      <c r="E108">
+        <v>2017</v>
+      </c>
+      <c r="F108" t="s">
+        <v>235</v>
+      </c>
+      <c r="G108" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A109" t="s">
+        <v>266</v>
+      </c>
+      <c r="B109" t="s">
+        <v>253</v>
+      </c>
+      <c r="C109" t="s">
+        <v>254</v>
+      </c>
+      <c r="D109" t="s">
+        <v>186</v>
+      </c>
+      <c r="E109">
+        <v>2013</v>
+      </c>
+      <c r="F109" t="s">
+        <v>235</v>
+      </c>
+      <c r="G109" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A110" t="s">
+        <v>267</v>
+      </c>
+      <c r="B110" t="s">
+        <v>253</v>
+      </c>
+      <c r="C110" t="s">
+        <v>255</v>
+      </c>
+      <c r="D110" t="s">
+        <v>186</v>
+      </c>
+      <c r="E110">
+        <v>2015</v>
+      </c>
+      <c r="F110" t="s">
+        <v>235</v>
+      </c>
+      <c r="G110" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A111" t="s">
+        <v>268</v>
+      </c>
+      <c r="B111" t="s">
+        <v>260</v>
+      </c>
+      <c r="C111" t="s">
+        <v>259</v>
+      </c>
+      <c r="D111" t="s">
+        <v>204</v>
+      </c>
+      <c r="E111">
+        <v>1982</v>
+      </c>
+      <c r="F111" t="s">
+        <v>261</v>
+      </c>
+      <c r="G111" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A112" t="s">
+        <v>269</v>
+      </c>
+      <c r="B112" t="s">
+        <v>3</v>
+      </c>
+      <c r="C112" t="s">
+        <v>270</v>
+      </c>
+      <c r="D112" t="s">
+        <v>271</v>
+      </c>
+      <c r="E112">
+        <v>2018</v>
+      </c>
+      <c r="F112" t="s">
+        <v>239</v>
+      </c>
+      <c r="G112" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A113" t="s">
+        <v>212</v>
+      </c>
+      <c r="B113" t="s">
+        <v>40</v>
+      </c>
+      <c r="C113" t="s">
+        <v>97</v>
+      </c>
+      <c r="D113" t="s">
+        <v>282</v>
+      </c>
+      <c r="E113">
+        <v>1962</v>
+      </c>
+      <c r="F113" t="s">
+        <v>239</v>
+      </c>
+      <c r="G113" t="s">
+        <v>243</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="B95:C95 A13:G94">
-    <cfRule type="expression" dxfId="1" priority="1">
+  <conditionalFormatting sqref="B111:C111 A28:G110 A15:G15 A1:G1 A3:G3 A5:G5 A7:G7 A9:G9 A11:G11 A13:G13">
+    <cfRule type="expression" dxfId="10" priority="10">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F3:G12 A95:A96 D95:G96 B96 A97:G97">
-    <cfRule type="expression" dxfId="0" priority="2">
+  <conditionalFormatting sqref="A111:A112 D111:G112 B112 A113:G113 F28:G28 F16:G16 F18:G18 F20:G20 F22:G22 F24:G24 F26:G26 F2:G2 F4:G4 F6:G6 F8:G8 F10:G10 F12:G12 F14:G14">
+    <cfRule type="expression" dxfId="9" priority="11">
+      <formula>MOD(ROW(),2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H17:I17">
+    <cfRule type="expression" dxfId="2" priority="3">
+      <formula>MOD(ROW(),2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A16:G27">
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>MOD(ROW(),2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:G2 A4:G4 A6:G6 A8:G8 A10:G10 A12:G12 A14:G14">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>